<commit_message>
docs: record M0-T1 approval; close ADR-002 (Fastify); update tracker/status
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2318A39F-1CE6-4D63-98FF-BAAB023A1804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{737005F2-2C45-4435-A5CB-E3118FA10134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{B18A36B0-3338-4466-9AB4-07C7B4EC695A}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{FAF2360E-8F85-449E-BDEB-472406CA6A27}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -85,13 +85,13 @@
     <t>Low blast radius; check boundary lint + reproducibility</t>
   </si>
   <si>
-    <t>D-002/D-003 approval</t>
-  </si>
-  <si>
-    <t>Blocked - awaiting PO approvals</t>
-  </si>
-  <si>
-    <t>Explicit PO go-ahead required before starting (founding-task gate)</t>
+    <t>ADR-002 (closed 2026-09-03)</t>
+  </si>
+  <si>
+    <t>Ready to start - approved by PO 2026-09-03</t>
+  </si>
+  <si>
+    <t>Branch m0-t1-scaffolding; Fastify decided (ADR-002); D-002/D-003 ratification still needed before M1</t>
   </si>
   <si>
     <t>M0-T2</t>
@@ -965,22 +965,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00551A40-E475-43A2-ADF3-BE01707981E3}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{00551A40-E475-43A2-ADF3-BE01707981E3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E6F3D0C0-DACA-4F94-9CF2-7ED3C7622FD7}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{E6F3D0C0-DACA-4F94-9CF2-7ED3C7622FD7}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{DE527B30-1D51-4E9F-9EBF-2E8F4B577BA4}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{C0A136B3-06FB-4515-9236-A5DC92E19103}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{65994BE6-082C-4DA9-9799-AF74387CEABB}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{3213EEDF-2142-4A7D-BF80-1E554A7270F9}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{E09E45F5-55A8-402F-99DB-D830D1ABD751}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{ADFB5838-0F7F-4E08-B585-204BED6C3177}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{57267A1A-2C78-443D-A4C1-46C1AC905684}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{5CFB04A8-8BD8-4ADA-AB03-DFE7FC08A376}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{4BA1A6A7-D483-4510-A28C-F2A5263CC97A}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{8A4D923E-E679-4B2F-85A5-288960290927}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{95F19405-8AC5-4AAB-A42C-C1CD00304DBB}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{8F3EDA31-1CD0-4A7F-9A1C-4578BE7789CF}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{965606ED-364B-4A6B-844E-49553A448D98}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{9ED15C2A-56BC-4D10-B20C-8B92C77D112D}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{71C438BD-B76A-419C-9964-80C0A12B3039}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{D44A4296-DBEA-4F32-9333-BF69FA0303F2}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{56A1F38C-9F4B-465E-9707-9A9FA87FC920}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{783BCE32-A8F5-4D3F-8BB1-5C0991A34F25}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{32E92550-9060-4FA2-8ED7-25616C8619AC}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{5F54D514-6810-4184-8E1A-D9BD8824030C}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{488EAEBC-99ED-49BF-B3D7-C969644A0FFC}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{2E70AB8E-2079-4875-AD69-44E2D0B54A58}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{1B53815D-9579-41F1-ADF5-3D8F9A71CD8B}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{C344D5D1-D043-4498-917E-6FB5A846D51F}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{2A6944D3-261F-4572-B288-441B3275438F}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{FB2A5EEF-32E7-4233-ADF1-0D8A3B126121}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1302,7 +1302,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7276CE-04E5-44A6-9E72-39BF2DDFF7FA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5328099B-5474-46DB-9074-3CBB7716C64F}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1316,7 +1316,7 @@
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
     <col min="10" max="10" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="39" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
   </cols>
@@ -1947,9 +1947,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept M0-T1 (reviewed, merged) - status/backlog/tracker updates
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{737005F2-2C45-4435-A5CB-E3118FA10134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D2F866A-3376-4898-AB43-05AE61E792AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{FAF2360E-8F85-449E-BDEB-472406CA6A27}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{35D1D25F-C3E1-443E-8549-C00C08940C61}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="116">
   <si>
     <t>ID</t>
   </si>
@@ -88,10 +88,13 @@
     <t>ADR-002 (closed 2026-09-03)</t>
   </si>
   <si>
-    <t>Ready to start - approved by PO 2026-09-03</t>
-  </si>
-  <si>
-    <t>Branch m0-t1-scaffolding; Fastify decided (ADR-002); D-002/D-003 ratification still needed before M1</t>
+    <t>Done - accepted &amp; merged 2026-09-03</t>
+  </si>
+  <si>
+    <t>Sonnet worker / Sonnet reviewer</t>
+  </si>
+  <si>
+    <t>Review: PASS WITH FIXES (.gitattributes + release-age comment); fixes applied &amp; re-verified at acceptance</t>
   </si>
   <si>
     <t>M0-T2</t>
@@ -965,22 +968,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E6F3D0C0-DACA-4F94-9CF2-7ED3C7622FD7}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{E6F3D0C0-DACA-4F94-9CF2-7ED3C7622FD7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D3AF356D-7B93-495D-853D-ADD0F9FD6215}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{D3AF356D-7B93-495D-853D-ADD0F9FD6215}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{9ED15C2A-56BC-4D10-B20C-8B92C77D112D}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{71C438BD-B76A-419C-9964-80C0A12B3039}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{D44A4296-DBEA-4F32-9333-BF69FA0303F2}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{56A1F38C-9F4B-465E-9707-9A9FA87FC920}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{783BCE32-A8F5-4D3F-8BB1-5C0991A34F25}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{32E92550-9060-4FA2-8ED7-25616C8619AC}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{5F54D514-6810-4184-8E1A-D9BD8824030C}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{488EAEBC-99ED-49BF-B3D7-C969644A0FFC}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{2E70AB8E-2079-4875-AD69-44E2D0B54A58}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{1B53815D-9579-41F1-ADF5-3D8F9A71CD8B}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{C344D5D1-D043-4498-917E-6FB5A846D51F}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{2A6944D3-261F-4572-B288-441B3275438F}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{FB2A5EEF-32E7-4233-ADF1-0D8A3B126121}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D842716F-20BE-44C2-B946-5E8DAB749C22}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{F14AE819-297D-4FDB-AB46-A90EFF170119}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{36C92D6C-41C7-4C8B-BFF9-61657AA3400D}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{A7AA7C7D-7A17-4048-96DA-C7EE4BC5BE4F}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{280D56F5-BDD5-4E83-8BC0-EF4B6417D569}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{3B09F9AE-29D8-449F-9C16-A5E074C9CCC0}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{9A79278B-1E51-4A72-A3E5-50AE16D1F7A3}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{F35426DE-330B-44A9-A985-8E9EE74F19E2}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{B4AFD439-7EDA-4548-9D46-4D544632A70A}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{B7C79994-66D7-458C-B33C-67FBA2814060}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{CE7F40FC-C6E9-4281-868A-BA519D0AAFC1}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{82ED1317-9344-4296-AB6D-7BF6699EC3F9}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{5BA9DFDA-DAAA-4A29-85A6-C5E6621707A9}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1302,7 +1305,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5328099B-5474-46DB-9074-3CBB7716C64F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06CC1EAC-B545-44B0-B390-07A7664DE51F}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1316,8 +1319,8 @@
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
     <col min="10" max="10" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1396,14 +1399,16 @@
       <c r="K2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="1"/>
+      <c r="L2" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="M2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>14</v>
@@ -1412,7 +1417,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>17</v>
@@ -1421,115 +1426,115 @@
         <v>18</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="I4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="1"/>
       <c r="M4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>17</v>
@@ -1538,76 +1543,76 @@
         <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>17</v>
@@ -1616,333 +1621,333 @@
         <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="I9" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: dispatch M0-T2 (CI) - ticket amended for missing gh CLI
Verification via deliberate-failure demo branches + public Actions API;
branch protection delivered as owner checklist. Tracker/status updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D2F866A-3376-4898-AB43-05AE61E792AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9492ED2C-EE7E-46A4-AD36-49D7939C6214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{35D1D25F-C3E1-443E-8549-C00C08940C61}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E99A5D88-582E-42D0-BF45-D138728CB767}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="117">
   <si>
     <t>ID</t>
   </si>
@@ -103,40 +103,43 @@
     <t>CI pipeline &amp; quality gates</t>
   </si>
   <si>
-    <t>Standard CI config from stock actions; verified by deliberate-failure PRs</t>
-  </si>
-  <si>
-    <t>Self-demonstrating acceptance criteria; check gate coverage + branch protection</t>
-  </si>
-  <si>
-    <t>M0-T1; repo remote decision</t>
+    <t>Standard CI config from stock actions; verified by deliberate-failure branches</t>
+  </si>
+  <si>
+    <t>Self-demonstrating acceptance criteria; check gate coverage + protection checklist</t>
+  </si>
+  <si>
+    <t>M0-T1 (done); GitHub remote (done)</t>
+  </si>
+  <si>
+    <t>Dispatched - in progress 2026-09-08</t>
+  </si>
+  <si>
+    <t>Branch m0-t2-ci; gh CLI absent so branch protection = owner checklist; ticket amended 2026-09-08</t>
+  </si>
+  <si>
+    <t>M1-T1</t>
+  </si>
+  <si>
+    <t>M1 Domain + inventory ledger</t>
+  </si>
+  <si>
+    <t>M1-E1 Deterministic domain package</t>
+  </si>
+  <si>
+    <t>Inventory ledger core</t>
+  </si>
+  <si>
+    <t>Opus</t>
+  </si>
+  <si>
+    <t>Highest-risk domain work: ledger/reconciliation math + idempotency + immutability</t>
+  </si>
+  <si>
+    <t>INV-LEDGER-1..4 are permanent guarantees; adversarial review of derivation/replay/negative-qty</t>
   </si>
   <si>
     <t>Not started</t>
-  </si>
-  <si>
-    <t>OneDrive/remote decision needed first (see STATUS.md)</t>
-  </si>
-  <si>
-    <t>M1-T1</t>
-  </si>
-  <si>
-    <t>M1 Domain + inventory ledger</t>
-  </si>
-  <si>
-    <t>M1-E1 Deterministic domain package</t>
-  </si>
-  <si>
-    <t>Inventory ledger core</t>
-  </si>
-  <si>
-    <t>Opus</t>
-  </si>
-  <si>
-    <t>Highest-risk domain work: ledger/reconciliation math + idempotency + immutability</t>
-  </si>
-  <si>
-    <t>INV-LEDGER-1..4 are permanent guarantees; adversarial review of derivation/replay/negative-qty</t>
   </si>
   <si>
     <t>Property tests INV-LEDGER-1..4 required</t>
@@ -968,22 +971,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D3AF356D-7B93-495D-853D-ADD0F9FD6215}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{D3AF356D-7B93-495D-853D-ADD0F9FD6215}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CE31D596-8EB9-4A87-89CD-F558332F9632}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{CE31D596-8EB9-4A87-89CD-F558332F9632}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{D842716F-20BE-44C2-B946-5E8DAB749C22}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{F14AE819-297D-4FDB-AB46-A90EFF170119}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{36C92D6C-41C7-4C8B-BFF9-61657AA3400D}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{A7AA7C7D-7A17-4048-96DA-C7EE4BC5BE4F}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{280D56F5-BDD5-4E83-8BC0-EF4B6417D569}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{3B09F9AE-29D8-449F-9C16-A5E074C9CCC0}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{9A79278B-1E51-4A72-A3E5-50AE16D1F7A3}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{F35426DE-330B-44A9-A985-8E9EE74F19E2}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{B4AFD439-7EDA-4548-9D46-4D544632A70A}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{B7C79994-66D7-458C-B33C-67FBA2814060}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{CE7F40FC-C6E9-4281-868A-BA519D0AAFC1}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{82ED1317-9344-4296-AB6D-7BF6699EC3F9}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{5BA9DFDA-DAAA-4A29-85A6-C5E6621707A9}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{114FFBBF-351D-4D6D-91B9-DA21B4B309D0}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{79732533-C849-4893-B284-912B2AFFE056}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{B57E4C70-FB96-47E5-B340-12DF83ABEA4B}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{2B493DE9-BCD9-41F0-80B9-CF04BE6FDD64}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{DF49BE2D-AAAF-4067-B64E-6AA76DBAD2A4}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{095253D1-2F9C-412A-89F8-C453D528EDB5}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{908C39B7-4DDA-49E7-9E75-A245BB62C49B}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{6AA804A5-59A2-4BD1-B1D0-856E42C450FA}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{EFC7722D-C99A-4F05-847F-29B3C5AD0FB4}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{5C77C7B1-ED8F-4103-B91B-5CCA2D2696CC}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{BD2C15AD-8143-4F04-9FFD-A7CF356D7761}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{2DB6F8EC-5A72-43C5-A27C-F144CF2D40A9}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{D93E5122-3E36-49FD-95C8-23C75FE16FB8}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1305,7 +1308,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06CC1EAC-B545-44B0-B390-07A7664DE51F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E29C6A-E1FB-4B2B-87B4-6B6C39CB7C46}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1318,7 +1321,7 @@
     <col min="7" max="7" width="50.7109375" customWidth="1"/>
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
-    <col min="10" max="10" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="34.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="29.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
@@ -1440,7 +1443,9 @@
       <c r="K3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="1"/>
+      <c r="L3" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="M3" s="1" t="s">
         <v>31</v>
       </c>
@@ -1477,16 +1482,16 @@
         <v>13</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L4" s="1"/>
       <c r="M4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>33</v>
@@ -1495,7 +1500,7 @@
         <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>17</v>
@@ -1504,28 +1509,28 @@
         <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>33</v>
@@ -1534,7 +1539,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>17</v>
@@ -1543,28 +1548,28 @@
         <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>33</v>
@@ -1573,7 +1578,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>17</v>
@@ -1582,37 +1587,37 @@
         <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>17</v>
@@ -1621,333 +1626,333 @@
         <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="I9" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: D-016 foundation-first - ratify D-003/ADR-008, unblock M1
PO directive (2026-09-08): build non-UI foundation now. Ledger decision
DECIDED; M1 tickets unblocked as scope-invariant. D-002 (MVP cut)
remains PROPOSED and now gates M3 (UI) + M5+ sequencing instead of M1.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9492ED2C-EE7E-46A4-AD36-49D7939C6214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D1011B4-7DC7-467F-94FA-48B09027D6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E99A5D88-582E-42D0-BF45-D138728CB767}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8857A009-93E7-49C1-B972-64D0BAECF582}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="121">
   <si>
     <t>ID</t>
   </si>
@@ -139,103 +139,115 @@
     <t>INV-LEDGER-1..4 are permanent guarantees; adversarial review of derivation/replay/negative-qty</t>
   </si>
   <si>
+    <t>M0-T1 (done)</t>
+  </si>
+  <si>
+    <t>Ready - unblocked 2026-09-08 (D-016)</t>
+  </si>
+  <si>
+    <t>Property tests INV-LEDGER-1..4 required</t>
+  </si>
+  <si>
+    <t>M1-T2</t>
+  </si>
+  <si>
+    <t>Postgres schema &amp; migrations (identity/household/inventory)</t>
+  </si>
+  <si>
+    <t>Sensitive schema for inventory history; append-only enforcement; tenancy/RLS</t>
+  </si>
+  <si>
+    <t>Isolation + append-only guarantees must survive adversarial review; migration reversibility</t>
+  </si>
+  <si>
+    <t>M1-T1; D-007</t>
+  </si>
+  <si>
+    <t>Blocked on M1-T1</t>
+  </si>
+  <si>
+    <t>RLS spike decision recorded in ADR-003</t>
+  </si>
+  <si>
+    <t>M1-T3</t>
+  </si>
+  <si>
+    <t>Units &amp; quantity model</t>
+  </si>
+  <si>
+    <t>Pure well-specified conversion functions with strong property tests</t>
+  </si>
+  <si>
+    <t>INV-SHOP-1 + nutrition math sit on this; silent conversion errors would corrupt inventory arithmetic</t>
+  </si>
+  <si>
+    <t>Never guess densities; typed IncompatibleUnits errors</t>
+  </si>
+  <si>
+    <t>M1-T4</t>
+  </si>
+  <si>
+    <t>Allergen rule engine (deterministic)</t>
+  </si>
+  <si>
+    <t>Safety-critical allergen enforcement (rule-23 high-risk list)</t>
+  </si>
+  <si>
+    <t>Adversarial review required (INV-ALRG-1/2); try to slip inputs past the screen</t>
+  </si>
+  <si>
+    <t>M0-T1 (done); fixtures from M1-T5</t>
+  </si>
+  <si>
+    <t>Ready - pair with M1-T5 fixtures</t>
+  </si>
+  <si>
+    <t>Output states: blocked / allowed-with-unknowns / allowed - never plain safe</t>
+  </si>
+  <si>
+    <t>M1-T5</t>
+  </si>
+  <si>
+    <t>M1-E2 Product knowledge foundations</t>
+  </si>
+  <si>
+    <t>Product lookup port + fixture adapter + coverage research spike</t>
+  </si>
+  <si>
+    <t>Adapter interfaces + fixture plumbing + read-only research script</t>
+  </si>
+  <si>
+    <t>Check port-boundary hygiene (no vendor types; provenance present) + research method</t>
+  </si>
+  <si>
+    <t>Feeds ADR-006 decision (R-1); no paid API signups without approval</t>
+  </si>
+  <si>
+    <t>M2</t>
+  </si>
+  <si>
+    <t>M2 Household + inventory API</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Auth integration + household/inventory endpoints + isolation suite</t>
+  </si>
+  <si>
+    <t>TBD at ticketing</t>
+  </si>
+  <si>
+    <t>Authz/tenancy tickets expected Opus; CRUD wiring Sonnet</t>
+  </si>
+  <si>
+    <t>Isolation tickets expected Opus review</t>
+  </si>
+  <si>
+    <t>M1</t>
+  </si>
+  <si>
     <t>Not started</t>
-  </si>
-  <si>
-    <t>Property tests INV-LEDGER-1..4 required</t>
-  </si>
-  <si>
-    <t>M1-T2</t>
-  </si>
-  <si>
-    <t>Postgres schema &amp; migrations (identity/household/inventory)</t>
-  </si>
-  <si>
-    <t>Sensitive schema for inventory history; append-only enforcement; tenancy/RLS</t>
-  </si>
-  <si>
-    <t>Isolation + append-only guarantees must survive adversarial review; migration reversibility</t>
-  </si>
-  <si>
-    <t>M1-T1; D-007</t>
-  </si>
-  <si>
-    <t>RLS spike decision recorded in ADR-003</t>
-  </si>
-  <si>
-    <t>M1-T3</t>
-  </si>
-  <si>
-    <t>Units &amp; quantity model</t>
-  </si>
-  <si>
-    <t>Pure well-specified conversion functions with strong property tests</t>
-  </si>
-  <si>
-    <t>INV-SHOP-1 + nutrition math sit on this; silent conversion errors would corrupt inventory arithmetic</t>
-  </si>
-  <si>
-    <t>Never guess densities; typed IncompatibleUnits errors</t>
-  </si>
-  <si>
-    <t>M1-T4</t>
-  </si>
-  <si>
-    <t>Allergen rule engine (deterministic)</t>
-  </si>
-  <si>
-    <t>Safety-critical allergen enforcement (rule-23 high-risk list)</t>
-  </si>
-  <si>
-    <t>Adversarial review required (INV-ALRG-1/2); try to slip inputs past the screen</t>
-  </si>
-  <si>
-    <t>M0-T1; fixtures from M1-T5</t>
-  </si>
-  <si>
-    <t>Output states: blocked / allowed-with-unknowns / allowed - never plain safe</t>
-  </si>
-  <si>
-    <t>M1-T5</t>
-  </si>
-  <si>
-    <t>M1-E2 Product knowledge foundations</t>
-  </si>
-  <si>
-    <t>Product lookup port + fixture adapter + coverage research spike</t>
-  </si>
-  <si>
-    <t>Adapter interfaces + fixture plumbing + read-only research script</t>
-  </si>
-  <si>
-    <t>Check port-boundary hygiene (no vendor types; provenance present) + research method</t>
-  </si>
-  <si>
-    <t>Feeds ADR-006 decision (R-1); no paid API signups without approval</t>
-  </si>
-  <si>
-    <t>M2</t>
-  </si>
-  <si>
-    <t>M2 Household + inventory API</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Auth integration + household/inventory endpoints + isolation suite</t>
-  </si>
-  <si>
-    <t>TBD at ticketing</t>
-  </si>
-  <si>
-    <t>Authz/tenancy tickets expected Opus; CRUD wiring Sonnet</t>
-  </si>
-  <si>
-    <t>Isolation tickets expected Opus review</t>
-  </si>
-  <si>
-    <t>M1</t>
   </si>
   <si>
     <t>Ticketed when M1 underway; contains cost-approval gates (auth vendor + PaaS)</t>
@@ -971,22 +983,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CE31D596-8EB9-4A87-89CD-F558332F9632}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{CE31D596-8EB9-4A87-89CD-F558332F9632}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CA4A944-F534-4AB2-99DF-EAAD292F7156}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{4CA4A944-F534-4AB2-99DF-EAAD292F7156}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{114FFBBF-351D-4D6D-91B9-DA21B4B309D0}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{79732533-C849-4893-B284-912B2AFFE056}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{B57E4C70-FB96-47E5-B340-12DF83ABEA4B}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{2B493DE9-BCD9-41F0-80B9-CF04BE6FDD64}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{DF49BE2D-AAAF-4067-B64E-6AA76DBAD2A4}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{095253D1-2F9C-412A-89F8-C453D528EDB5}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{908C39B7-4DDA-49E7-9E75-A245BB62C49B}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{6AA804A5-59A2-4BD1-B1D0-856E42C450FA}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{EFC7722D-C99A-4F05-847F-29B3C5AD0FB4}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{5C77C7B1-ED8F-4103-B91B-5CCA2D2696CC}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{BD2C15AD-8143-4F04-9FFD-A7CF356D7761}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{2DB6F8EC-5A72-43C5-A27C-F144CF2D40A9}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{D93E5122-3E36-49FD-95C8-23C75FE16FB8}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{03EC01B2-37AD-4B4B-B8E8-8C7DB8478ABB}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{8C36FD57-C27B-4FB9-8880-73C8DCB0ACB8}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{F9B659AD-7CCF-44FC-9B18-536761D6EE97}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{78F7447F-27DB-4233-830E-A3E51DB0867F}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{0399A7B1-350B-43BC-A893-8056C739DDF4}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{738D3001-23ED-471A-943D-63ACA942AE49}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{99485422-08F0-449C-994A-8885F15CD857}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{F066F8DF-2F07-4822-B370-9B8D80A1B4EA}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{3D058F15-B93A-4276-B313-71A3B0F38BB8}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{892569BB-018D-41D4-A5F6-B64DDC2FEFF4}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{8F96ECDC-C81F-466A-9AF9-917EDA449061}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{2E7764AF-FA3C-4E9C-9336-433BBC2EC4E4}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{E5112197-EAD1-43D5-B740-EF12FCEA052C}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1308,7 +1320,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E29C6A-E1FB-4B2B-87B4-6B6C39CB7C46}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{683645E5-D921-4011-A36E-67C0B25AA9D5}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1322,7 +1334,7 @@
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
     <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="29.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
   </cols>
@@ -1479,19 +1491,19 @@
         <v>38</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L4" s="1"/>
       <c r="M4" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>33</v>
@@ -1500,7 +1512,7 @@
         <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>17</v>
@@ -1509,28 +1521,28 @@
         <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>33</v>
@@ -1539,7 +1551,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>17</v>
@@ -1548,28 +1560,28 @@
         <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>33</v>
@@ -1578,7 +1590,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>17</v>
@@ -1587,37 +1599,37 @@
         <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>17</v>
@@ -1626,333 +1638,333 @@
         <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: accept M0-T2 (reviewed PASS, merged) - Milestone 0 complete
Deviation sign-off recorded; M0-T2 follow-ups triaged; stale README
lines refreshed; tracker/status updated. Next: M1-T1 dispatch +
owner applies branch-protection checklist.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D1011B4-7DC7-467F-94FA-48B09027D6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{958180DF-F6FB-4E3F-963A-88365062C939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8857A009-93E7-49C1-B972-64D0BAECF582}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6071259C-813E-4BA8-A440-802E474B5979}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -112,10 +112,10 @@
     <t>M0-T1 (done); GitHub remote (done)</t>
   </si>
   <si>
-    <t>Dispatched - in progress 2026-09-08</t>
-  </si>
-  <si>
-    <t>Branch m0-t2-ci; gh CLI absent so branch protection = owner checklist; ticket amended 2026-09-08</t>
+    <t>Done - accepted &amp; merged 2026-09-08</t>
+  </si>
+  <si>
+    <t>Review: PASS no fixes (runs re-verified via Actions API); deviation (pnpm version pinning) architect-approved; branch protection = owner checklist pending</t>
   </si>
   <si>
     <t>M1-T1</t>
@@ -983,22 +983,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CA4A944-F534-4AB2-99DF-EAAD292F7156}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{4CA4A944-F534-4AB2-99DF-EAAD292F7156}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E0980D65-83A2-467D-8DFF-6D60C39A8236}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{E0980D65-83A2-467D-8DFF-6D60C39A8236}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{03EC01B2-37AD-4B4B-B8E8-8C7DB8478ABB}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{8C36FD57-C27B-4FB9-8880-73C8DCB0ACB8}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{F9B659AD-7CCF-44FC-9B18-536761D6EE97}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{78F7447F-27DB-4233-830E-A3E51DB0867F}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{0399A7B1-350B-43BC-A893-8056C739DDF4}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{738D3001-23ED-471A-943D-63ACA942AE49}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{99485422-08F0-449C-994A-8885F15CD857}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{F066F8DF-2F07-4822-B370-9B8D80A1B4EA}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{3D058F15-B93A-4276-B313-71A3B0F38BB8}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{892569BB-018D-41D4-A5F6-B64DDC2FEFF4}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{8F96ECDC-C81F-466A-9AF9-917EDA449061}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{2E7764AF-FA3C-4E9C-9336-433BBC2EC4E4}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{E5112197-EAD1-43D5-B740-EF12FCEA052C}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{596FD9EC-FCAF-4061-A833-CAB6A5B9C745}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{B1C2FFAA-DEBF-4A89-BC2F-D0D6E3094F29}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{8E09DF81-A415-487A-A3A6-BFCB8CF88158}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{60771AD5-3D78-4B71-9243-FD1C17B4ADAD}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{930710C5-C03F-4DBA-B804-1EDFF3FF55BA}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{2AA31C94-256A-4A1F-A382-FA8F005DEB56}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{3C9328BA-03FD-4014-8B11-20C875A0F382}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{EBA894F3-98DD-461C-B01F-B2FBAEAFE474}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{1B85B6D2-E22B-40EF-BABB-17E8B0E48967}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{790AE63F-0893-4C34-9454-D363492EA9BB}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{D26A3F65-DB88-4BAE-85D9-2A50C217A31C}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{B1E7D02A-387A-4AD8-926A-6A76CD4683B3}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{D88992EB-7071-462F-BCA2-341D8EAD2900}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1320,7 +1320,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{683645E5-D921-4011-A36E-67C0B25AA9D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72A8E12-D248-48B9-BF96-964959FAC2D6}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1421,7 +1421,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
docs: codify dispatch & handoff convention (rules 28-30); dispatch M1-T1
Option A (architect-dispatched worker/reviewer sub-agents) + Option C
(handoff reports committed under docs/handoff/) per PO approval.
Current-phase note refreshed (M0 complete, M1 underway).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{958180DF-F6FB-4E3F-963A-88365062C939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{80CC8192-352D-4F80-ABC7-C2A1BFC29294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6071259C-813E-4BA8-A440-802E474B5979}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA7D7CA1-3B00-4086-9867-996F35457B48}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="123">
   <si>
     <t>ID</t>
   </si>
@@ -142,43 +142,49 @@
     <t>M0-T1 (done)</t>
   </si>
   <si>
+    <t>Dispatched - in progress 2026-09-08</t>
+  </si>
+  <si>
+    <t>Opus worker / Opus reviewer (architect-dispatched)</t>
+  </si>
+  <si>
+    <t>Branch m1-t1-ledger; property tests INV-LEDGER-1..4 required; handoff per CLAUDE.md rules 28-30</t>
+  </si>
+  <si>
+    <t>M1-T2</t>
+  </si>
+  <si>
+    <t>Postgres schema &amp; migrations (identity/household/inventory)</t>
+  </si>
+  <si>
+    <t>Sensitive schema for inventory history; append-only enforcement; tenancy/RLS</t>
+  </si>
+  <si>
+    <t>Isolation + append-only guarantees must survive adversarial review; migration reversibility</t>
+  </si>
+  <si>
+    <t>M1-T1; D-007</t>
+  </si>
+  <si>
+    <t>Blocked on M1-T1</t>
+  </si>
+  <si>
+    <t>RLS spike decision recorded in ADR-003</t>
+  </si>
+  <si>
+    <t>M1-T3</t>
+  </si>
+  <si>
+    <t>Units &amp; quantity model</t>
+  </si>
+  <si>
+    <t>Pure well-specified conversion functions with strong property tests</t>
+  </si>
+  <si>
+    <t>INV-SHOP-1 + nutrition math sit on this; silent conversion errors would corrupt inventory arithmetic</t>
+  </si>
+  <si>
     <t>Ready - unblocked 2026-09-08 (D-016)</t>
-  </si>
-  <si>
-    <t>Property tests INV-LEDGER-1..4 required</t>
-  </si>
-  <si>
-    <t>M1-T2</t>
-  </si>
-  <si>
-    <t>Postgres schema &amp; migrations (identity/household/inventory)</t>
-  </si>
-  <si>
-    <t>Sensitive schema for inventory history; append-only enforcement; tenancy/RLS</t>
-  </si>
-  <si>
-    <t>Isolation + append-only guarantees must survive adversarial review; migration reversibility</t>
-  </si>
-  <si>
-    <t>M1-T1; D-007</t>
-  </si>
-  <si>
-    <t>Blocked on M1-T1</t>
-  </si>
-  <si>
-    <t>RLS spike decision recorded in ADR-003</t>
-  </si>
-  <si>
-    <t>M1-T3</t>
-  </si>
-  <si>
-    <t>Units &amp; quantity model</t>
-  </si>
-  <si>
-    <t>Pure well-specified conversion functions with strong property tests</t>
-  </si>
-  <si>
-    <t>INV-SHOP-1 + nutrition math sit on this; silent conversion errors would corrupt inventory arithmetic</t>
   </si>
   <si>
     <t>Never guess densities; typed IncompatibleUnits errors</t>
@@ -983,22 +989,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E0980D65-83A2-467D-8DFF-6D60C39A8236}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{E0980D65-83A2-467D-8DFF-6D60C39A8236}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A6CAD3B4-314C-4748-BB0D-40AE958DE981}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{A6CAD3B4-314C-4748-BB0D-40AE958DE981}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{596FD9EC-FCAF-4061-A833-CAB6A5B9C745}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{B1C2FFAA-DEBF-4A89-BC2F-D0D6E3094F29}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{8E09DF81-A415-487A-A3A6-BFCB8CF88158}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{60771AD5-3D78-4B71-9243-FD1C17B4ADAD}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{930710C5-C03F-4DBA-B804-1EDFF3FF55BA}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{2AA31C94-256A-4A1F-A382-FA8F005DEB56}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{3C9328BA-03FD-4014-8B11-20C875A0F382}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{EBA894F3-98DD-461C-B01F-B2FBAEAFE474}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{1B85B6D2-E22B-40EF-BABB-17E8B0E48967}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{790AE63F-0893-4C34-9454-D363492EA9BB}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{D26A3F65-DB88-4BAE-85D9-2A50C217A31C}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{B1E7D02A-387A-4AD8-926A-6A76CD4683B3}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{D88992EB-7071-462F-BCA2-341D8EAD2900}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{E51E38AB-DAED-4D3F-A006-A2AAB54817FA}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{AB925D77-8067-46A1-9F81-DC9B6FE85425}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{DF70585F-A911-4A29-8F5B-6FC07E960AC7}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{70C546D6-0DFB-4DA9-A754-06E273AC0A0B}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{B45A749A-1737-48F7-BE8E-9BBEF900D73E}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{5D5D1420-CDF3-45EE-AC59-0564A7750CAE}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{3C23D4D8-CE64-4478-B28E-3EEF46923385}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{E6D5D14E-E7CF-482F-9B24-A39B2E9FEB3F}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{89C21B3A-637D-4F9F-9541-EAF250C18E83}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{42D34AE9-3232-4964-B39E-4205F949D635}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{C050BE25-7841-469E-8F2B-6EDE79F0996D}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{9873B4D0-7B2E-4A7A-85E7-35ACF9D3BCE1}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{79F78D5F-7ED4-4171-BBFB-78206AA63A20}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1320,7 +1326,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72A8E12-D248-48B9-BF96-964959FAC2D6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{490A375A-9983-4DF4-ADC2-7DB4520DB1E3}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1335,7 +1341,7 @@
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
     <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="47.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1496,14 +1502,16 @@
       <c r="K4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="L4" s="1"/>
+      <c r="L4" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="M4" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>33</v>
@@ -1512,7 +1520,7 @@
         <v>34</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>17</v>
@@ -1521,28 +1529,28 @@
         <v>36</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>33</v>
@@ -1551,7 +1559,7 @@
         <v>34</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>17</v>
@@ -1560,28 +1568,28 @@
         <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>39</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>33</v>
@@ -1590,7 +1598,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>17</v>
@@ -1599,37 +1607,37 @@
         <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>17</v>
@@ -1638,333 +1646,333 @@
         <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>39</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: accept M1-T1 - review record, settled semantics into docs, dispatch M1-T3
Commits docs/handoff/M1-T1.review.md; applies the worker-proposed
domain-model updates (exact-arithmetic ledger row, clamp invariant,
idempotency conflict semantics, OQ-1 narrowing); restates INV-LEDGER-4;
D-003 implementation addenda; ADR-010 timestamp note; M1-T2 acceptance
additions; follow-ups triaged; tracker/status updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80CC8192-352D-4F80-ABC7-C2A1BFC29294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A253629-C42E-4CD3-81D4-CA04BE3C3F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA7D7CA1-3B00-4086-9867-996F35457B48}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BE3BFBCA-CEF6-4E24-921C-E08AAC40A9F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="125">
   <si>
     <t>ID</t>
   </si>
@@ -142,88 +142,94 @@
     <t>M0-T1 (done)</t>
   </si>
   <si>
+    <t>Done - accepted &amp; squash-merged 2026-09-08</t>
+  </si>
+  <si>
+    <t>Opus worker / Opus reviewer (architect-dispatched)</t>
+  </si>
+  <si>
+    <t>Review: PASS after one fix round (forged-flag + rehydration trust closed; mutation-proven); 75 tests; handoff docs/handoff/M1-T1.*</t>
+  </si>
+  <si>
+    <t>M1-T2</t>
+  </si>
+  <si>
+    <t>Postgres schema &amp; migrations (identity/household/inventory)</t>
+  </si>
+  <si>
+    <t>Sensitive schema for inventory history; append-only enforcement; tenancy/RLS</t>
+  </si>
+  <si>
+    <t>Isolation + append-only guarantees must survive adversarial review; migration reversibility</t>
+  </si>
+  <si>
+    <t>M1-T1; D-007</t>
+  </si>
+  <si>
+    <t>Blocked on M1-T1</t>
+  </si>
+  <si>
+    <t>RLS spike decision recorded in ADR-003</t>
+  </si>
+  <si>
+    <t>M1-T3</t>
+  </si>
+  <si>
+    <t>Units &amp; quantity model</t>
+  </si>
+  <si>
+    <t>Pure well-specified conversion functions with strong property tests</t>
+  </si>
+  <si>
+    <t>INV-SHOP-1 + nutrition math sit on this; silent conversion errors would corrupt inventory arithmetic</t>
+  </si>
+  <si>
     <t>Dispatched - in progress 2026-09-08</t>
   </si>
   <si>
-    <t>Opus worker / Opus reviewer (architect-dispatched)</t>
-  </si>
-  <si>
-    <t>Branch m1-t1-ledger; property tests INV-LEDGER-1..4 required; handoff per CLAUDE.md rules 28-30</t>
-  </si>
-  <si>
-    <t>M1-T2</t>
-  </si>
-  <si>
-    <t>Postgres schema &amp; migrations (identity/household/inventory)</t>
-  </si>
-  <si>
-    <t>Sensitive schema for inventory history; append-only enforcement; tenancy/RLS</t>
-  </si>
-  <si>
-    <t>Isolation + append-only guarantees must survive adversarial review; migration reversibility</t>
-  </si>
-  <si>
-    <t>M1-T1; D-007</t>
-  </si>
-  <si>
-    <t>Blocked on M1-T1</t>
-  </si>
-  <si>
-    <t>RLS spike decision recorded in ADR-003</t>
-  </si>
-  <si>
-    <t>M1-T3</t>
-  </si>
-  <si>
-    <t>Units &amp; quantity model</t>
-  </si>
-  <si>
-    <t>Pure well-specified conversion functions with strong property tests</t>
-  </si>
-  <si>
-    <t>INV-SHOP-1 + nutrition math sit on this; silent conversion errors would corrupt inventory arithmetic</t>
+    <t>Sonnet worker / Opus reviewer (architect-dispatched)</t>
+  </si>
+  <si>
+    <t>Branch m1-t3-units; never guess densities; typed IncompatibleUnits errors</t>
+  </si>
+  <si>
+    <t>M1-T4</t>
+  </si>
+  <si>
+    <t>Allergen rule engine (deterministic)</t>
+  </si>
+  <si>
+    <t>Safety-critical allergen enforcement (rule-23 high-risk list)</t>
+  </si>
+  <si>
+    <t>Adversarial review required (INV-ALRG-1/2); try to slip inputs past the screen</t>
+  </si>
+  <si>
+    <t>M0-T1 (done); fixtures from M1-T5</t>
+  </si>
+  <si>
+    <t>Ready - pair with M1-T5 fixtures</t>
+  </si>
+  <si>
+    <t>Output states: blocked / allowed-with-unknowns / allowed - never plain safe</t>
+  </si>
+  <si>
+    <t>M1-T5</t>
+  </si>
+  <si>
+    <t>M1-E2 Product knowledge foundations</t>
+  </si>
+  <si>
+    <t>Product lookup port + fixture adapter + coverage research spike</t>
+  </si>
+  <si>
+    <t>Adapter interfaces + fixture plumbing + read-only research script</t>
+  </si>
+  <si>
+    <t>Check port-boundary hygiene (no vendor types; provenance present) + research method</t>
   </si>
   <si>
     <t>Ready - unblocked 2026-09-08 (D-016)</t>
-  </si>
-  <si>
-    <t>Never guess densities; typed IncompatibleUnits errors</t>
-  </si>
-  <si>
-    <t>M1-T4</t>
-  </si>
-  <si>
-    <t>Allergen rule engine (deterministic)</t>
-  </si>
-  <si>
-    <t>Safety-critical allergen enforcement (rule-23 high-risk list)</t>
-  </si>
-  <si>
-    <t>Adversarial review required (INV-ALRG-1/2); try to slip inputs past the screen</t>
-  </si>
-  <si>
-    <t>M0-T1 (done); fixtures from M1-T5</t>
-  </si>
-  <si>
-    <t>Ready - pair with M1-T5 fixtures</t>
-  </si>
-  <si>
-    <t>Output states: blocked / allowed-with-unknowns / allowed - never plain safe</t>
-  </si>
-  <si>
-    <t>M1-T5</t>
-  </si>
-  <si>
-    <t>M1-E2 Product knowledge foundations</t>
-  </si>
-  <si>
-    <t>Product lookup port + fixture adapter + coverage research spike</t>
-  </si>
-  <si>
-    <t>Adapter interfaces + fixture plumbing + read-only research script</t>
-  </si>
-  <si>
-    <t>Check port-boundary hygiene (no vendor types; provenance present) + research method</t>
   </si>
   <si>
     <t>Feeds ADR-006 decision (R-1); no paid API signups without approval</t>
@@ -989,22 +995,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A6CAD3B4-314C-4748-BB0D-40AE958DE981}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{A6CAD3B4-314C-4748-BB0D-40AE958DE981}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{177CAFE0-F401-4E85-B023-5AD496395742}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{177CAFE0-F401-4E85-B023-5AD496395742}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{E51E38AB-DAED-4D3F-A006-A2AAB54817FA}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{AB925D77-8067-46A1-9F81-DC9B6FE85425}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{DF70585F-A911-4A29-8F5B-6FC07E960AC7}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{70C546D6-0DFB-4DA9-A754-06E273AC0A0B}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{B45A749A-1737-48F7-BE8E-9BBEF900D73E}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{5D5D1420-CDF3-45EE-AC59-0564A7750CAE}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{3C23D4D8-CE64-4478-B28E-3EEF46923385}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{E6D5D14E-E7CF-482F-9B24-A39B2E9FEB3F}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{89C21B3A-637D-4F9F-9541-EAF250C18E83}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{42D34AE9-3232-4964-B39E-4205F949D635}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{C050BE25-7841-469E-8F2B-6EDE79F0996D}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{9873B4D0-7B2E-4A7A-85E7-35ACF9D3BCE1}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{79F78D5F-7ED4-4171-BBFB-78206AA63A20}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{1DB5EB9B-C6DE-4A1A-9CC5-78BD3BA8CF03}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{AC8A5512-B71B-4098-BC06-8D731DE27590}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{E69D37EA-074E-458F-9557-2D0211828278}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{26A93B40-8DE4-47C3-B3E1-22E49F868A5B}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{7A6EE90A-F819-43B3-AF09-29CBD7CA2FC6}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{E3EDCF41-302B-402B-8F23-A009D5FCEF29}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{9CE0B346-2684-412E-908F-ADECF77A1C22}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{234471A5-F65A-4178-80BB-C842D1AAB1A0}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{F178A6E1-EB93-40C3-B6F2-32B30D1DE318}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{0CE97110-6D94-4B50-B33C-136D35F21B47}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{8C61CAB9-B9E1-408D-8AC3-7D9DC510950A}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{72BF33ED-B837-431D-8FFF-1110AED41711}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{338EDA1C-1BDC-45F6-8839-A21FC43D9B6B}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1326,7 +1332,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{490A375A-9983-4DF4-ADC2-7DB4520DB1E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE561FB-FC72-4E44-B43E-BD159510B858}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1340,8 +1346,8 @@
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
     <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="47.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1468,7 +1474,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
@@ -1582,14 +1588,16 @@
       <c r="K6" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="L6" s="1"/>
+      <c r="L6" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="M6" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>33</v>
@@ -1598,7 +1606,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>17</v>
@@ -1607,37 +1615,37 @@
         <v>36</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>36</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>17</v>
@@ -1646,333 +1654,333 @@
         <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>39</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: accept M1-T3 - review record, OQ-2 resolved, dispatch M1-T5
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A253629-C42E-4CD3-81D4-CA04BE3C3F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9433EDDA-8A7F-47F9-B035-A837486973C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BE3BFBCA-CEF6-4E24-921C-E08AAC40A9F7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50B3D77C-D166-46C2-A494-A17876D96CCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="126">
   <si>
     <t>ID</t>
   </si>
@@ -184,13 +184,13 @@
     <t>INV-SHOP-1 + nutrition math sit on this; silent conversion errors would corrupt inventory arithmetic</t>
   </si>
   <si>
-    <t>Dispatched - in progress 2026-09-08</t>
+    <t>Done - accepted &amp; squash-merged 2026-09-09</t>
   </si>
   <si>
     <t>Sonnet worker / Opus reviewer (architect-dispatched)</t>
   </si>
   <si>
-    <t>Branch m1-t3-units; never guess densities; typed IncompatibleUnits errors</t>
+    <t>Review: PASS after one fix round (ground-truth factor pins added; makeBridge/alias/comparator defects closed); 150 tests</t>
   </si>
   <si>
     <t>M1-T4</t>
@@ -229,10 +229,13 @@
     <t>Check port-boundary hygiene (no vendor types; provenance present) + research method</t>
   </si>
   <si>
-    <t>Ready - unblocked 2026-09-08 (D-016)</t>
-  </si>
-  <si>
-    <t>Feeds ADR-006 decision (R-1); no paid API signups without approval</t>
+    <t>Dispatched - in progress 2026-09-09</t>
+  </si>
+  <si>
+    <t>Sonnet worker / Sonnet reviewer (architect-dispatched)</t>
+  </si>
+  <si>
+    <t>Branch m1-t5-product-lookup; feeds ADR-006 (R-1); no paid API signups</t>
   </si>
   <si>
     <t>M2</t>
@@ -995,22 +998,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{177CAFE0-F401-4E85-B023-5AD496395742}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{177CAFE0-F401-4E85-B023-5AD496395742}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BEEFF639-920D-4293-82F8-958B5061C4F8}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{BEEFF639-920D-4293-82F8-958B5061C4F8}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{1DB5EB9B-C6DE-4A1A-9CC5-78BD3BA8CF03}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{AC8A5512-B71B-4098-BC06-8D731DE27590}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{E69D37EA-074E-458F-9557-2D0211828278}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{26A93B40-8DE4-47C3-B3E1-22E49F868A5B}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{7A6EE90A-F819-43B3-AF09-29CBD7CA2FC6}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{E3EDCF41-302B-402B-8F23-A009D5FCEF29}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{9CE0B346-2684-412E-908F-ADECF77A1C22}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{234471A5-F65A-4178-80BB-C842D1AAB1A0}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{F178A6E1-EB93-40C3-B6F2-32B30D1DE318}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{0CE97110-6D94-4B50-B33C-136D35F21B47}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{8C61CAB9-B9E1-408D-8AC3-7D9DC510950A}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{72BF33ED-B837-431D-8FFF-1110AED41711}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{338EDA1C-1BDC-45F6-8839-A21FC43D9B6B}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{5C79DBFB-518E-4DE7-857F-A5CDC0A84F19}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{3024E01B-F322-4CB3-86D4-BDC3961EDDE9}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{6DD165C0-53E0-47C7-8416-A73B30AE5577}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{7715D170-169D-44B8-B971-CEB6204FEF75}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{D59075F0-36F1-4E06-855F-3D575CE2834C}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{8DC8B0A4-A3F3-498D-8498-321188E3F34A}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{A36CAE97-0C19-4234-ACDD-E25761EBE78B}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{9CFBD7E6-5677-4D12-A1A6-020CEECCE1EB}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{E5E57BD0-816F-4F25-9268-1B4C5F2FE5BB}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{26EE4F10-0B87-48DA-BEDF-3B14F85D046D}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{0FD109A2-C20E-4F4B-A094-C1EF8730F3D9}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{1F1DA2DB-3DD6-4282-B5D8-07919C71C4FB}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{A7A00B22-A5F0-481B-B8DF-2061930C7D36}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1332,7 +1335,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FE561FB-FC72-4E44-B43E-BD159510B858}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03DE3EB-3DFD-42D5-B96F-820961FE56AF}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1347,7 +1350,7 @@
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
     <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="50.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1554,7 +1557,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>50</v>
       </c>
@@ -1668,319 +1671,321 @@
       <c r="K8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="L8" s="1"/>
+      <c r="L8" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="M8" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>75</v>
-      </c>
       <c r="I9" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: accept M1-T5 - review record, ADR-006 OPEN -> PROPOSED (R-1), dispatch M1-T4
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9433EDDA-8A7F-47F9-B035-A837486973C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E196905-4C28-4E87-899A-DB4853AA8FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50B3D77C-D166-46C2-A494-A17876D96CCF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B8DFF34-D81E-4A58-B2C9-DEA4DBE11240}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="125">
   <si>
     <t>ID</t>
   </si>
@@ -205,13 +205,13 @@
     <t>Adversarial review required (INV-ALRG-1/2); try to slip inputs past the screen</t>
   </si>
   <si>
-    <t>M0-T1 (done); fixtures from M1-T5</t>
-  </si>
-  <si>
-    <t>Ready - pair with M1-T5 fixtures</t>
-  </si>
-  <si>
-    <t>Output states: blocked / allowed-with-unknowns / allowed - never plain safe</t>
+    <t>M0-T1 (done); fixtures from M1-T5 (done)</t>
+  </si>
+  <si>
+    <t>Dispatched - in progress 2026-09-09</t>
+  </si>
+  <si>
+    <t>Branch m1-t4-allergens; output states: blocked / allowed-with-unknowns / allowed - never plain safe</t>
   </si>
   <si>
     <t>M1-T5</t>
@@ -229,13 +229,10 @@
     <t>Check port-boundary hygiene (no vendor types; provenance present) + research method</t>
   </si>
   <si>
-    <t>Dispatched - in progress 2026-09-09</t>
-  </si>
-  <si>
     <t>Sonnet worker / Sonnet reviewer (architect-dispatched)</t>
   </si>
   <si>
-    <t>Branch m1-t5-product-lookup; feeds ADR-006 (R-1); no paid API signups</t>
+    <t>Review: PASS after doc-only fixes; R-1 delivered; ADR-006 -&gt; PROPOSED; 216 tests</t>
   </si>
   <si>
     <t>M2</t>
@@ -998,22 +995,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BEEFF639-920D-4293-82F8-958B5061C4F8}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{BEEFF639-920D-4293-82F8-958B5061C4F8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{507B7820-A84F-4839-8C38-67A638A45AC8}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{507B7820-A84F-4839-8C38-67A638A45AC8}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{5C79DBFB-518E-4DE7-857F-A5CDC0A84F19}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{3024E01B-F322-4CB3-86D4-BDC3961EDDE9}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{6DD165C0-53E0-47C7-8416-A73B30AE5577}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{7715D170-169D-44B8-B971-CEB6204FEF75}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{D59075F0-36F1-4E06-855F-3D575CE2834C}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{8DC8B0A4-A3F3-498D-8498-321188E3F34A}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{A36CAE97-0C19-4234-ACDD-E25761EBE78B}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{9CFBD7E6-5677-4D12-A1A6-020CEECCE1EB}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{E5E57BD0-816F-4F25-9268-1B4C5F2FE5BB}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{26EE4F10-0B87-48DA-BEDF-3B14F85D046D}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{0FD109A2-C20E-4F4B-A094-C1EF8730F3D9}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{1F1DA2DB-3DD6-4282-B5D8-07919C71C4FB}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{A7A00B22-A5F0-481B-B8DF-2061930C7D36}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{EA97AA1E-086C-4037-A4C1-ED964CB49419}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{B112FE0E-CD20-491C-B6F8-AF6F7F8FB629}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{9688882D-E5EA-4580-BD14-13ADED5E4EFD}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{0BC4A134-3FE5-42BA-9875-7B8A849118AC}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{5363B15A-C745-42B7-9281-68B24140953A}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{4247B55B-3D5A-4DD6-BBAD-1DCD99A375BD}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{E21F93C8-965E-4279-9CC6-81F08D7F41AF}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{0840C5D9-C35A-4CD0-8D47-3E74B7EEBBD4}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{DF3921A9-AD3B-4674-88BB-F617330AC1C6}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{F194BD44-8216-4AEA-B174-5ADB4B2AFBB2}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{5F2B7811-581F-4721-B1EE-C93E46ACEF98}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{8B035A4A-DCEF-4499-92BE-1DBB8939FD61}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{DEEEF049-4950-43BC-A42F-87AE84E262B8}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1335,7 +1332,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03DE3EB-3DFD-42D5-B96F-820961FE56AF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA7E0D2-30A2-409E-A1BE-011A3F3EF1AD}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1348,7 +1345,7 @@
     <col min="7" max="7" width="50.7109375" customWidth="1"/>
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
-    <col min="10" max="10" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="37.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="42.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="50.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
@@ -1632,7 +1629,9 @@
       <c r="K7" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="L7" s="1"/>
+      <c r="L7" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="M7" s="1" t="s">
         <v>63</v>
       </c>
@@ -1669,323 +1668,323 @@
         <v>39</v>
       </c>
       <c r="K8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="M8" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>86</v>
-      </c>
       <c r="J10" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="K11" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G12" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="K12" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G13" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="J13" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="K13" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="J14" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G15" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>119</v>
-      </c>
       <c r="J15" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>122</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G16" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>124</v>
-      </c>
       <c r="J16" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L16" s="1"/>
       <c r="M16" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: accept M1-T4 - review record, D-017 policies, aggregation invariant, dispatch M1-T2
AllergenDeclaration + assertion-kind notes and worst-wins invariant 8
into domain-model; recommendations-fixture mirror note into
testing-strategy; UI copy rules bound to M3/M6 epics; mandatory pre-M4
gates + follow-ups triaged; M1-T2 amended for missing Docker
(DATABASE_URL-gated tests + CI Postgres service container).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E196905-4C28-4E87-899A-DB4853AA8FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9028E0E2-FA13-4303-909B-C20C7C91A5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B8DFF34-D81E-4A58-B2C9-DEA4DBE11240}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89C95BDD-68EA-4895-87DC-1D94FB588664}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="125">
   <si>
     <t>ID</t>
   </si>
@@ -163,13 +163,13 @@
     <t>Isolation + append-only guarantees must survive adversarial review; migration reversibility</t>
   </si>
   <si>
-    <t>M1-T1; D-007</t>
-  </si>
-  <si>
-    <t>Blocked on M1-T1</t>
-  </si>
-  <si>
-    <t>RLS spike decision recorded in ADR-003</t>
+    <t>M1-T1 (done); D-007</t>
+  </si>
+  <si>
+    <t>Dispatched - in progress 2026-09-10</t>
+  </si>
+  <si>
+    <t>Branch m1-t2-schema; amended for missing Docker (DATABASE_URL-gated tests + CI service container); RLS spike decision to ADR-003</t>
   </si>
   <si>
     <t>M1-T3</t>
@@ -208,10 +208,10 @@
     <t>M0-T1 (done); fixtures from M1-T5 (done)</t>
   </si>
   <si>
-    <t>Dispatched - in progress 2026-09-09</t>
-  </si>
-  <si>
-    <t>Branch m1-t4-allergens; output states: blocked / allowed-with-unknowns / allowed - never plain safe</t>
+    <t>Done - accepted &amp; squash-merged 2026-09-10</t>
+  </si>
+  <si>
+    <t>Review: PASS after one fix round (3 fail-open paths to ALLOWED closed; mutation-pinned); 163 tests; policies D-017</t>
   </si>
   <si>
     <t>M1-T5</t>
@@ -995,22 +995,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{507B7820-A84F-4839-8C38-67A638A45AC8}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{507B7820-A84F-4839-8C38-67A638A45AC8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{47280937-4703-4F24-A418-7C8A9E84F78B}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M16" xr:uid="{47280937-4703-4F24-A418-7C8A9E84F78B}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{EA97AA1E-086C-4037-A4C1-ED964CB49419}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{B112FE0E-CD20-491C-B6F8-AF6F7F8FB629}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{9688882D-E5EA-4580-BD14-13ADED5E4EFD}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{0BC4A134-3FE5-42BA-9875-7B8A849118AC}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{5363B15A-C745-42B7-9281-68B24140953A}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{4247B55B-3D5A-4DD6-BBAD-1DCD99A375BD}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{E21F93C8-965E-4279-9CC6-81F08D7F41AF}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{0840C5D9-C35A-4CD0-8D47-3E74B7EEBBD4}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{DF3921A9-AD3B-4674-88BB-F617330AC1C6}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{F194BD44-8216-4AEA-B174-5ADB4B2AFBB2}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{5F2B7811-581F-4721-B1EE-C93E46ACEF98}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{8B035A4A-DCEF-4499-92BE-1DBB8939FD61}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{DEEEF049-4950-43BC-A42F-87AE84E262B8}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{5D614576-C452-49ED-9669-99DCCF5F8F19}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{9E3E20E3-A549-41E7-8A9E-20EE293AD0FA}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{C5A8AF4B-F341-491C-B58E-821AD22D0FF6}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{A972A873-C018-4D41-AC8F-4EA9B2A44978}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{64886C57-45B1-4F49-A8C9-CC6672EEA52D}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{05508533-4734-44E6-A74A-02E74BDB0B7F}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{61A16E38-2305-47A1-ABAD-49D6DCBB515A}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{B52053A8-6013-458F-A097-53C580F159A9}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{32686A81-EE39-4133-A095-A90D439010DA}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{60F3FEFA-630A-4DD4-AB1C-FCA72FD54377}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{2D2D2FC0-16B5-4F9B-80F6-05E1BFC70878}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{BD4F5143-D30C-4680-9703-6BEAB7B4AD84}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{0D2A6534-D21C-4DCD-A95F-5245AB4E6BAD}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1332,7 +1332,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA7E0D2-30A2-409E-A1BE-011A3F3EF1AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15D78A61-8340-40B4-922E-6631ACF00ECC}">
   <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1515,7 +1515,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
@@ -1549,7 +1549,9 @@
       <c r="K5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="L5" s="1"/>
+      <c r="L5" s="1" t="s">
+        <v>41</v>
+      </c>
       <c r="M5" s="1" t="s">
         <v>49</v>
       </c>
@@ -1595,7 +1597,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>57</v>
       </c>

</xml_diff>

<commit_message>
docs: accept M1-T2 - MILESTONE 1 COMPLETE; ADR-003 DECIDED, ADR-008 closed
Review record committed; standing schema rules (household-scoped unique
constraints, SECURITY DEFINER for RLS-reading triggers, security_invoker
views) recorded in ADR-003; data-model implementation notes; follow-ups
triaged incl. M2-blocking definer-owner role; status/tracker updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TRACKER.xlsx
+++ b/BACKLOG_TRACKER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/006_Smart Kitchen App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9028E0E2-FA13-4303-909B-C20C7C91A5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8605058C-B97B-4573-A6BA-828763F845F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89C95BDD-68EA-4895-87DC-1D94FB588664}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{169DF65E-B017-4D24-8B36-1507841430F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="134">
   <si>
     <t>ID</t>
   </si>
@@ -166,10 +166,10 @@
     <t>M1-T1 (done); D-007</t>
   </si>
   <si>
-    <t>Dispatched - in progress 2026-09-10</t>
-  </si>
-  <si>
-    <t>Branch m1-t2-schema; amended for missing Docker (DATABASE_URL-gated tests + CI service container); RLS spike decision to ADR-003</t>
+    <t>Done - accepted &amp; squash-merged 2026-09-10 - MILESTONE 1 COMPLETE</t>
+  </si>
+  <si>
+    <t>Review: PASS after one fix round (INV-LEDGER-4 fail-open + unique-index oracle closed; worker self-found CREATE ROLE race); 96 DB tests; ADR-003 DECIDED</t>
   </si>
   <si>
     <t>M1-T3</t>
@@ -265,12 +265,39 @@
     <t>Ticketed when M1 underway; contains cost-approval gates (auth vendor + PaaS)</t>
   </si>
   <si>
+    <t>M3-E0</t>
+  </si>
+  <si>
+    <t>M3 Basic client inventory experience</t>
+  </si>
+  <si>
+    <t>UX design gate: wireframes + hi-fi mockups + safety-copy deck + validation</t>
+  </si>
+  <si>
+    <t>Sonnet-class design work</t>
+  </si>
+  <si>
+    <t>Design docs/mockups only - no code (PO directive 2026-09-10)</t>
+  </si>
+  <si>
+    <t>PO review</t>
+  </si>
+  <si>
+    <t>PO + Dean on-device review + hallway test are the review</t>
+  </si>
+  <si>
+    <t>M1 (done); design-direction + ux-plan docs</t>
+  </si>
+  <si>
+    <t>Ready - awaiting PO kickoff</t>
+  </si>
+  <si>
+    <t>Exit gate: PO sign-off + D-002 ratified before M3 build tickets exist</t>
+  </si>
+  <si>
     <t>M3</t>
   </si>
   <si>
-    <t>M3 Basic client inventory experience</t>
-  </si>
-  <si>
     <t>Expo app: auth/household/inventory/barcode confirm flow</t>
   </si>
   <si>
@@ -280,7 +307,7 @@
     <t>Sonnet expected; provenance-badge UX reviewed vs PRD</t>
   </si>
   <si>
-    <t>Correction-rate telemetry goes live here</t>
+    <t>Correction-rate telemetry goes live here; GATED by new M3-E0 UX-design epic (docs/design/ux-plan.md) + D-002</t>
   </si>
   <si>
     <t>M4</t>
@@ -995,22 +1022,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{47280937-4703-4F24-A418-7C8A9E84F78B}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M16" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:M16" xr:uid="{47280937-4703-4F24-A418-7C8A9E84F78B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{09C2DA67-EDD6-4018-B030-834156A6F019}" name="BacklogTracker" displayName="BacklogTracker" ref="A1:M17" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:M17" xr:uid="{09C2DA67-EDD6-4018-B030-834156A6F019}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{5D614576-C452-49ED-9669-99DCCF5F8F19}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{9E3E20E3-A549-41E7-8A9E-20EE293AD0FA}" name="Milestone" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{C5A8AF4B-F341-491C-B58E-821AD22D0FF6}" name="Epic" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{A972A873-C018-4D41-AC8F-4EA9B2A44978}" name="Title" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{64886C57-45B1-4F49-A8C9-CC6672EEA52D}" name="Type" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{05508533-4734-44E6-A74A-02E74BDB0B7F}" name="Impl Model" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{61A16E38-2305-47A1-ABAD-49D6DCBB515A}" name="Impl Model Reason" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{B52053A8-6013-458F-A097-53C580F159A9}" name="Review Model" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{32686A81-EE39-4133-A095-A90D439010DA}" name="Review Model Reason" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{60F3FEFA-630A-4DD4-AB1C-FCA72FD54377}" name="Dependencies" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{2D2D2FC0-16B5-4F9B-80F6-05E1BFC70878}" name="Status" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{BD4F5143-D30C-4680-9703-6BEAB7B4AD84}" name="Assignee" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{0D2A6534-D21C-4DCD-A95F-5245AB4E6BAD}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{C001EF29-C496-4FCE-8D61-05234827E770}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{5A97686B-80DB-43C9-AB13-8EBD82E47B8A}" name="Milestone" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{7B75FE7E-A2FB-4CD5-B56F-68DD52958013}" name="Epic" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{B039C296-FFAC-431B-826C-846E1FFD555C}" name="Title" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{A5D297A7-3B26-471D-BA29-C9BD26196E2D}" name="Type" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{64C59427-B3D5-4184-80D5-53D5858854A1}" name="Impl Model" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{6BD18526-AE46-401E-B314-BC8D5002D234}" name="Impl Model Reason" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{12A03C6B-778F-497C-8627-2EC93DF9B946}" name="Review Model" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{1CF494FD-3528-4207-9893-EDFE281DDA9A}" name="Review Model Reason" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{16CE54AB-3072-48A9-A72E-744405838911}" name="Dependencies" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{45DD0305-2974-402E-9CFC-69AD3D8D5B8C}" name="Status" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{C1E6FB66-FF47-4BA5-BC1F-645891CFC07A}" name="Assignee" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{9DE93D7F-0F55-4725-986C-6957AC3BDA83}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1332,21 +1359,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15D78A61-8340-40B4-922E-6631ACF00ECC}">
-  <dimension ref="A1:M16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E448F88A-DB55-459A-9021-79F076CAEE6A}">
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="63" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="50.7109375" customWidth="1"/>
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" customWidth="1"/>
-    <col min="10" max="10" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="65.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="50.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50.7109375" customWidth="1"/>
   </cols>
@@ -1735,40 +1762,40 @@
         <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>73</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>2</v>
@@ -1777,37 +1804,37 @@
         <v>75</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>75</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>79</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>73</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>2</v>
@@ -1816,37 +1843,37 @@
         <v>75</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>75</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>79</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>73</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>2</v>
@@ -1855,37 +1882,37 @@
         <v>75</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>75</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>79</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>73</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>2</v>
@@ -1894,37 +1921,37 @@
         <v>75</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>75</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>79</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>73</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>2</v>
@@ -1933,35 +1960,37 @@
         <v>75</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>75</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>79</v>
       </c>
       <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
+      <c r="M15" s="1" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>73</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>2</v>
@@ -1970,23 +1999,60 @@
         <v>75</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>75</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>79</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="M16" s="1" t="s">
-        <v>124</v>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>